<commit_message>
Update problem hanlde when login failed
</commit_message>
<xml_diff>
--- a/TestBrand.xlsx
+++ b/TestBrand.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chenzhijun/GithubProject/Twitter-Scraper-Script/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Vscode\Twitter-Scraper-Script\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9ECCA9D-0A48-744D-B83F-BF21463354FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C92AD157-930C-4181-8823-ED9AA64442F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="37920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>@Apple</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>@Nike</t>
   </si>
@@ -47,13 +44,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -364,17 +361,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G100"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G99"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.1640625" customWidth="1"/>
+    <col min="1" max="1" width="18.125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="7" max="7" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -382,7 +379,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -392,7 +389,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -402,10 +399,8 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -774,11 +769,6 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="1"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
-      <c r="F50" s="1"/>
-      <c r="G50" s="1"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" s="1"/>
@@ -926,9 +916,6 @@
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A99" s="1"/>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>